<commit_message>
Update variable name closes #229
</commit_message>
<xml_diff>
--- a/data/epp-16-ns-data.xlsx
+++ b/data/epp-16-ns-data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gavin.brown/Desktop/rst-test-specs/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gavin.brown/Code/rst-test-specs/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FC7DC3-D749-A94E-B64A-AEB2FD410C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933420EB-7FF3-C044-B19B-FDDDEC83CA27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{CD472396-4CFB-9A45-AA99-46F4E9CB8B91}"/>
   </bookViews>
@@ -202,21 +202,6 @@
     <t>EPP_DOMAIN_UPDATE_SERVER_ACCEPTS_HOST_ATTRIBUTES_WITHOUT_GLUE</t>
   </si>
   <si>
-    <t>{"ns2.epp-16.rst." &amp; $name}</t>
-  </si>
-  <si>
-    <t>{"ns3.epp-16.rst." &amp; $name}</t>
-  </si>
-  <si>
-    <t>{"ns4.epp-16.rst." &amp; $name}</t>
-  </si>
-  <si>
-    <t>{"ns5.epp-16.rst." &amp; $name}</t>
-  </si>
-  <si>
-    <t>{"ns6.epp-16.rst." &amp; $name}</t>
-  </si>
-  <si>
     <t>ipType</t>
   </si>
   <si>
@@ -224,6 +209,21 @@
   </si>
   <si>
     <t>IP address to add (if any)</t>
+  </si>
+  <si>
+    <t>{"ns2.epp-16.rst." &amp; $DOMAIN}</t>
+  </si>
+  <si>
+    <t>{"ns3.epp-16.rst." &amp; $DOMAIN}</t>
+  </si>
+  <si>
+    <t>{"ns4.epp-16.rst." &amp; $DOMAIN}</t>
+  </si>
+  <si>
+    <t>{"ns5.epp-16.rst." &amp; $DOMAIN}</t>
+  </si>
+  <si>
+    <t>{"ns6.epp-16.rst." &amp; $DOMAIN}</t>
   </si>
 </sst>
 </file>
@@ -975,7 +975,7 @@
         <v>12</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>30</v>
@@ -999,10 +999,10 @@
         <v>15</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>4</v>
@@ -1200,7 +1200,7 @@
         <v>10</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>1</v>
@@ -1228,7 +1228,7 @@
     </row>
     <row r="21" spans="3:9" x14ac:dyDescent="0.2">
       <c r="E21" s="5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>28</v>
@@ -1346,7 +1346,7 @@
     </row>
     <row r="29" spans="3:9" x14ac:dyDescent="0.2">
       <c r="E29" s="5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>39</v>
@@ -1363,7 +1363,7 @@
     </row>
     <row r="30" spans="3:9" x14ac:dyDescent="0.2">
       <c r="E30" s="5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>41</v>
@@ -1380,7 +1380,7 @@
     </row>
     <row r="31" spans="3:9" x14ac:dyDescent="0.2">
       <c r="E31" s="5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>41</v>

</xml_diff>